<commit_message>
Welches t test to tables
</commit_message>
<xml_diff>
--- a/output/tables/spo2_12h_by_treatment_obs.xlsx
+++ b/output/tables/spo2_12h_by_treatment_obs.xlsx
@@ -12,13 +12,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">Time Since Randomisation (hours)
 </t>
   </si>
   <si>
     <t xml:space="preserve">Mean (SD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welch Two Sample t-test</t>
   </si>
   <si>
     <t xml:space="preserve">Observations
@@ -99,6 +102,13 @@
   </si>
   <si>
     <t xml:space="preserve">94.05 (3.18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p-value
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;0.001</t>
   </si>
 </sst>
 </file>
@@ -539,6 +549,7 @@
     <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="10.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="NA" customHeight="1">
@@ -546,13 +557,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="NA" customHeight="1">
@@ -563,10 +577,13 @@
         <v>409</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="NA" customHeight="1">
@@ -577,10 +594,13 @@
         <v>689</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="NA" customHeight="1">
@@ -591,10 +611,13 @@
         <v>683</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5" ht="NA" customHeight="1">
@@ -605,10 +628,13 @@
         <v>681</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6" ht="NA" customHeight="1">
@@ -619,10 +645,13 @@
         <v>697</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7" ht="NA" customHeight="1">
@@ -633,10 +662,13 @@
         <v>660</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" ht="NA" customHeight="1">
@@ -647,10 +679,13 @@
         <v>664</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9" ht="NA" customHeight="1">
@@ -661,10 +696,13 @@
         <v>618</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10" ht="NA" customHeight="1">
@@ -675,10 +713,13 @@
         <v>563</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="11" ht="NA" customHeight="1">
@@ -689,10 +730,13 @@
         <v>523</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="12" ht="NA" customHeight="1">
@@ -703,10 +747,13 @@
         <v>525</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="13" ht="NA" customHeight="1">
@@ -722,10 +769,31 @@
       <c r="D13" s="5" t="s">
         <v>1</v>
       </c>
+      <c r="E13" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="NA" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A13:D13"/>
+  <mergeCells count="2">
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>